<commit_message>
docs: adicionar modificacoes MP080 repo
</commit_message>
<xml_diff>
--- a/areas_land_bank_com_id.xlsx
+++ b/areas_land_bank_com_id.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="EsteLivro" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matias.matos\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinicius.castro\Documents\01 Profissional\Buriti Empreendimentos\Repositórios\teste-mapa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D48CF6A0-E11B-49C6-B37A-49B3A2E21D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76EF4B67-BB62-434F-8E42-066A3FE04D67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{2D7381EB-1656-47BB-A82F-14AB3B13CCCD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2D7381EB-1656-47BB-A82F-14AB3B13CCCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2354" uniqueCount="712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2354" uniqueCount="706">
   <si>
     <t>Nome</t>
   </si>
@@ -1858,24 +1858,6 @@
     <t>MAP013</t>
   </si>
   <si>
-    <t>MAP014</t>
-  </si>
-  <si>
-    <t>MAP015</t>
-  </si>
-  <si>
-    <t>MAP016</t>
-  </si>
-  <si>
-    <t>MAP017</t>
-  </si>
-  <si>
-    <t>MAP018</t>
-  </si>
-  <si>
-    <t>MAP019</t>
-  </si>
-  <si>
     <t>MAP020</t>
   </si>
   <si>
@@ -2050,139 +2032,139 @@
     <t>MAP079</t>
   </si>
   <si>
+    <t>MAP082</t>
+  </si>
+  <si>
+    <t>MAP083</t>
+  </si>
+  <si>
+    <t>MAP084</t>
+  </si>
+  <si>
+    <t>MAP085</t>
+  </si>
+  <si>
+    <t>MAP086</t>
+  </si>
+  <si>
+    <t>MAP087</t>
+  </si>
+  <si>
+    <t>MAP088</t>
+  </si>
+  <si>
+    <t>MAP089</t>
+  </si>
+  <si>
+    <t>MAP090</t>
+  </si>
+  <si>
+    <t>MAP091</t>
+  </si>
+  <si>
+    <t>MAP092</t>
+  </si>
+  <si>
+    <t>MAP093</t>
+  </si>
+  <si>
+    <t>MAP094</t>
+  </si>
+  <si>
+    <t>MAP095</t>
+  </si>
+  <si>
+    <t>MAP096</t>
+  </si>
+  <si>
+    <t>MAP097</t>
+  </si>
+  <si>
+    <t>MAP098</t>
+  </si>
+  <si>
+    <t>MAP099</t>
+  </si>
+  <si>
+    <t>MAP100</t>
+  </si>
+  <si>
+    <t>MAP101</t>
+  </si>
+  <si>
+    <t>MAP102</t>
+  </si>
+  <si>
+    <t>MAP103</t>
+  </si>
+  <si>
+    <t>MAP104</t>
+  </si>
+  <si>
+    <t>MAP105</t>
+  </si>
+  <si>
+    <t>MAP106</t>
+  </si>
+  <si>
+    <t>MAP107</t>
+  </si>
+  <si>
+    <t>MAP108</t>
+  </si>
+  <si>
+    <t>MAP109</t>
+  </si>
+  <si>
+    <t>MAP110</t>
+  </si>
+  <si>
+    <t>MAP111</t>
+  </si>
+  <si>
+    <t>MAP112</t>
+  </si>
+  <si>
+    <t>MAP113</t>
+  </si>
+  <si>
+    <t>MAP114</t>
+  </si>
+  <si>
+    <t>MAP115</t>
+  </si>
+  <si>
+    <t>MAP116</t>
+  </si>
+  <si>
+    <t>MAP117</t>
+  </si>
+  <si>
+    <t>MAP118</t>
+  </si>
+  <si>
+    <t>MAP119</t>
+  </si>
+  <si>
+    <t>MAP120</t>
+  </si>
+  <si>
+    <t>MAP121</t>
+  </si>
+  <si>
+    <t>MAP122</t>
+  </si>
+  <si>
+    <t>MAP027</t>
+  </si>
+  <si>
+    <t>MAP050</t>
+  </si>
+  <si>
+    <t>MAP081</t>
+  </si>
+  <si>
     <t>MAP080</t>
-  </si>
-  <si>
-    <t>MAP081</t>
-  </si>
-  <si>
-    <t>MAP082</t>
-  </si>
-  <si>
-    <t>MAP083</t>
-  </si>
-  <si>
-    <t>MAP084</t>
-  </si>
-  <si>
-    <t>MAP085</t>
-  </si>
-  <si>
-    <t>MAP086</t>
-  </si>
-  <si>
-    <t>MAP087</t>
-  </si>
-  <si>
-    <t>MAP088</t>
-  </si>
-  <si>
-    <t>MAP089</t>
-  </si>
-  <si>
-    <t>MAP090</t>
-  </si>
-  <si>
-    <t>MAP091</t>
-  </si>
-  <si>
-    <t>MAP092</t>
-  </si>
-  <si>
-    <t>MAP093</t>
-  </si>
-  <si>
-    <t>MAP094</t>
-  </si>
-  <si>
-    <t>MAP095</t>
-  </si>
-  <si>
-    <t>MAP096</t>
-  </si>
-  <si>
-    <t>MAP097</t>
-  </si>
-  <si>
-    <t>MAP098</t>
-  </si>
-  <si>
-    <t>MAP099</t>
-  </si>
-  <si>
-    <t>MAP100</t>
-  </si>
-  <si>
-    <t>MAP101</t>
-  </si>
-  <si>
-    <t>MAP102</t>
-  </si>
-  <si>
-    <t>MAP103</t>
-  </si>
-  <si>
-    <t>MAP104</t>
-  </si>
-  <si>
-    <t>MAP105</t>
-  </si>
-  <si>
-    <t>MAP106</t>
-  </si>
-  <si>
-    <t>MAP107</t>
-  </si>
-  <si>
-    <t>MAP108</t>
-  </si>
-  <si>
-    <t>MAP109</t>
-  </si>
-  <si>
-    <t>MAP110</t>
-  </si>
-  <si>
-    <t>MAP111</t>
-  </si>
-  <si>
-    <t>MAP112</t>
-  </si>
-  <si>
-    <t>MAP113</t>
-  </si>
-  <si>
-    <t>MAP114</t>
-  </si>
-  <si>
-    <t>MAP115</t>
-  </si>
-  <si>
-    <t>MAP116</t>
-  </si>
-  <si>
-    <t>MAP117</t>
-  </si>
-  <si>
-    <t>MAP118</t>
-  </si>
-  <si>
-    <t>MAP119</t>
-  </si>
-  <si>
-    <t>MAP120</t>
-  </si>
-  <si>
-    <t>MAP121</t>
-  </si>
-  <si>
-    <t>MAP122</t>
-  </si>
-  <si>
-    <t>MAP027</t>
-  </si>
-  <si>
-    <t>MAP050</t>
   </si>
 </sst>
 </file>
@@ -2780,37 +2762,37 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BB1E7F9-B7E0-4EE5-A96E-08F27078CA81}">
   <sheetPr codeName="Folha1"/>
   <dimension ref="A1:AW231"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="59.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.81640625" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="27.453125" style="27" customWidth="1"/>
-    <col min="5" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="42.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.7265625" customWidth="1"/>
+    <col min="2" max="2" width="59.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.77734375" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="27.44140625" style="27" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="42.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.77734375" customWidth="1"/>
     <col min="20" max="21" width="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="28" max="29" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="7.77734375" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="9" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.44140625" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="9" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="7" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="40" max="49" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="40" max="49" width="6.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" ht="65" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:49" ht="66" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>589</v>
       </c>
@@ -2959,7 +2941,7 @@
         <v>2035</v>
       </c>
     </row>
-    <row r="2" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>590</v>
       </c>
@@ -3106,7 +3088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>597</v>
       </c>
@@ -3247,7 +3229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A4" s="33" t="s">
         <v>598</v>
       </c>
@@ -3388,7 +3370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="33" t="s">
         <v>598</v>
       </c>
@@ -3529,7 +3511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>599</v>
       </c>
@@ -3670,7 +3652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>600</v>
       </c>
@@ -3811,7 +3793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>600</v>
       </c>
@@ -3952,7 +3934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>600</v>
       </c>
@@ -4093,7 +4075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>600</v>
       </c>
@@ -4234,7 +4216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>600</v>
       </c>
@@ -4375,7 +4357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>591</v>
       </c>
@@ -4516,7 +4498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>592</v>
       </c>
@@ -4657,7 +4639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>593</v>
       </c>
@@ -4798,7 +4780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>593</v>
       </c>
@@ -4939,7 +4921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>594</v>
       </c>
@@ -5080,7 +5062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>595</v>
       </c>
@@ -5221,7 +5203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>596</v>
       </c>
@@ -5362,7 +5344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>601</v>
       </c>
@@ -5503,7 +5485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>602</v>
       </c>
@@ -5644,9 +5626,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B21" s="20" t="s">
         <v>291</v>
@@ -5785,9 +5767,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B22" s="20" t="s">
         <v>292</v>
@@ -5926,9 +5908,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="B23" s="20" t="s">
         <v>293</v>
@@ -6067,9 +6049,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="B24" s="20" t="s">
         <v>294</v>
@@ -6208,9 +6190,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>607</v>
+        <v>602</v>
       </c>
       <c r="B25" s="20" t="s">
         <v>295</v>
@@ -6349,9 +6331,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>608</v>
+        <v>602</v>
       </c>
       <c r="B26" s="20" t="s">
         <v>296</v>
@@ -6490,9 +6472,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>609</v>
+        <v>603</v>
       </c>
       <c r="B27" s="20" t="s">
         <v>297</v>
@@ -6631,9 +6613,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B28" s="20" t="s">
         <v>298</v>
@@ -6772,9 +6754,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B29" s="20" t="s">
         <v>299</v>
@@ -6913,9 +6895,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B30" s="20" t="s">
         <v>300</v>
@@ -7054,9 +7036,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B31" s="20" t="s">
         <v>301</v>
@@ -7195,9 +7177,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B32" s="20" t="s">
         <v>302</v>
@@ -7336,9 +7318,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B33" s="20" t="s">
         <v>303</v>
@@ -7477,9 +7459,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B34" s="20" t="s">
         <v>304</v>
@@ -7618,9 +7600,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B35" s="20" t="s">
         <v>305</v>
@@ -7759,9 +7741,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B36" s="20" t="s">
         <v>306</v>
@@ -7900,9 +7882,9 @@
         <v>800</v>
       </c>
     </row>
-    <row r="37" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B37" s="20" t="s">
         <v>307</v>
@@ -8041,9 +8023,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B38" s="20" t="s">
         <v>308</v>
@@ -8182,9 +8164,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B39" s="20" t="s">
         <v>309</v>
@@ -8323,9 +8305,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B40" s="20" t="s">
         <v>310</v>
@@ -8464,9 +8446,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B41" s="20" t="s">
         <v>311</v>
@@ -8605,9 +8587,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B42" s="20" t="s">
         <v>312</v>
@@ -8746,9 +8728,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B43" s="20" t="s">
         <v>313</v>
@@ -8887,9 +8869,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B44" s="20" t="s">
         <v>314</v>
@@ -9028,9 +9010,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B45" s="20" t="s">
         <v>315</v>
@@ -9169,9 +9151,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="B46" s="20" t="s">
         <v>316</v>
@@ -9310,9 +9292,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>611</v>
+        <v>605</v>
       </c>
       <c r="B47" s="22" t="s">
         <v>577</v>
@@ -9457,9 +9439,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>611</v>
+        <v>605</v>
       </c>
       <c r="B48" s="22" t="s">
         <v>578</v>
@@ -9604,9 +9586,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>611</v>
+        <v>605</v>
       </c>
       <c r="B49" s="22" t="s">
         <v>317</v>
@@ -9751,9 +9733,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>611</v>
+        <v>605</v>
       </c>
       <c r="B50" s="22" t="s">
         <v>318</v>
@@ -9898,9 +9880,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>612</v>
+        <v>606</v>
       </c>
       <c r="B51" s="20" t="s">
         <v>319</v>
@@ -10039,9 +10021,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>614</v>
+        <v>608</v>
       </c>
       <c r="B52" s="4" t="s">
         <v>574</v>
@@ -10180,9 +10162,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>615</v>
+        <v>609</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>575</v>
@@ -10321,9 +10303,9 @@
         <v>360</v>
       </c>
     </row>
-    <row r="54" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>613</v>
+        <v>607</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>576</v>
@@ -10462,9 +10444,9 @@
         <v>380</v>
       </c>
     </row>
-    <row r="55" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>710</v>
+        <v>702</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>320</v>
@@ -10603,9 +10585,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>616</v>
+        <v>610</v>
       </c>
       <c r="B56" s="20" t="s">
         <v>321</v>
@@ -10744,9 +10726,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>618</v>
+        <v>612</v>
       </c>
       <c r="B57" s="20" t="s">
         <v>322</v>
@@ -10891,9 +10873,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>618</v>
+        <v>612</v>
       </c>
       <c r="B58" s="20" t="s">
         <v>323</v>
@@ -11038,9 +11020,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>617</v>
+        <v>611</v>
       </c>
       <c r="B59" s="20" t="s">
         <v>324</v>
@@ -11185,9 +11167,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>619</v>
+        <v>613</v>
       </c>
       <c r="B60" s="20" t="s">
         <v>325</v>
@@ -11332,9 +11314,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>620</v>
+        <v>614</v>
       </c>
       <c r="B61" s="20" t="s">
         <v>326</v>
@@ -11479,9 +11461,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>620</v>
+        <v>614</v>
       </c>
       <c r="B62" s="20" t="s">
         <v>327</v>
@@ -11626,9 +11608,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>621</v>
+        <v>615</v>
       </c>
       <c r="B63" s="20" t="s">
         <v>328</v>
@@ -11773,9 +11755,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>622</v>
+        <v>616</v>
       </c>
       <c r="B64" s="20" t="s">
         <v>329</v>
@@ -11914,9 +11896,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>622</v>
+        <v>616</v>
       </c>
       <c r="B65" s="20" t="s">
         <v>330</v>
@@ -12055,9 +12037,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>622</v>
+        <v>616</v>
       </c>
       <c r="B66" s="20" t="s">
         <v>331</v>
@@ -12196,9 +12178,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>623</v>
+        <v>617</v>
       </c>
       <c r="B67" s="20" t="s">
         <v>332</v>
@@ -12337,9 +12319,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>624</v>
+        <v>618</v>
       </c>
       <c r="B68" s="20" t="s">
         <v>333</v>
@@ -12478,9 +12460,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>625</v>
+        <v>619</v>
       </c>
       <c r="B69" s="20" t="s">
         <v>334</v>
@@ -12619,9 +12601,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>625</v>
+        <v>619</v>
       </c>
       <c r="B70" s="20" t="s">
         <v>334</v>
@@ -12760,9 +12742,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>626</v>
+        <v>620</v>
       </c>
       <c r="B71" s="20" t="s">
         <v>335</v>
@@ -12907,9 +12889,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>627</v>
+        <v>621</v>
       </c>
       <c r="B72" s="20" t="s">
         <v>336</v>
@@ -13054,9 +13036,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>627</v>
+        <v>621</v>
       </c>
       <c r="B73" s="20" t="s">
         <v>337</v>
@@ -13201,9 +13183,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>628</v>
+        <v>622</v>
       </c>
       <c r="B74" s="20" t="s">
         <v>338</v>
@@ -13348,9 +13330,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>628</v>
+        <v>622</v>
       </c>
       <c r="B75" s="20" t="s">
         <v>339</v>
@@ -13495,9 +13477,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>629</v>
+        <v>623</v>
       </c>
       <c r="B76" s="20" t="s">
         <v>340</v>
@@ -13642,9 +13624,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>629</v>
+        <v>623</v>
       </c>
       <c r="B77" s="20" t="s">
         <v>341</v>
@@ -13789,9 +13771,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
       <c r="B78" s="20" t="s">
         <v>342</v>
@@ -13936,9 +13918,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
       <c r="B79" s="20" t="s">
         <v>343</v>
@@ -14083,9 +14065,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
       <c r="B80" s="20" t="s">
         <v>344</v>
@@ -14230,9 +14212,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>631</v>
+        <v>625</v>
       </c>
       <c r="B81" s="20" t="s">
         <v>345</v>
@@ -14377,9 +14359,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>631</v>
+        <v>625</v>
       </c>
       <c r="B82" s="20" t="s">
         <v>346</v>
@@ -14524,9 +14506,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>632</v>
+        <v>626</v>
       </c>
       <c r="B83" s="20" t="s">
         <v>347</v>
@@ -14671,9 +14653,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>633</v>
+        <v>627</v>
       </c>
       <c r="B84" s="20" t="s">
         <v>348</v>
@@ -14818,9 +14800,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>634</v>
+        <v>628</v>
       </c>
       <c r="B85" s="20" t="s">
         <v>349</v>
@@ -14965,9 +14947,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>634</v>
+        <v>628</v>
       </c>
       <c r="B86" s="20" t="s">
         <v>350</v>
@@ -15112,9 +15094,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>634</v>
+        <v>628</v>
       </c>
       <c r="B87" s="20" t="s">
         <v>351</v>
@@ -15259,9 +15241,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>635</v>
+        <v>629</v>
       </c>
       <c r="B88" s="20" t="s">
         <v>352</v>
@@ -15406,9 +15388,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>636</v>
+        <v>630</v>
       </c>
       <c r="B89" s="20" t="s">
         <v>353</v>
@@ -15553,9 +15535,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>636</v>
+        <v>630</v>
       </c>
       <c r="B90" s="20" t="s">
         <v>354</v>
@@ -15700,9 +15682,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>637</v>
+        <v>631</v>
       </c>
       <c r="B91" s="20" t="s">
         <v>355</v>
@@ -15847,9 +15829,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="B92" s="20" t="s">
         <v>356</v>
@@ -15994,9 +15976,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>638</v>
+        <v>632</v>
       </c>
       <c r="B93" s="20" t="s">
         <v>357</v>
@@ -16141,9 +16123,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>638</v>
+        <v>632</v>
       </c>
       <c r="B94" s="20" t="s">
         <v>358</v>
@@ -16288,9 +16270,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>638</v>
+        <v>632</v>
       </c>
       <c r="B95" s="20" t="s">
         <v>359</v>
@@ -16435,9 +16417,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>638</v>
+        <v>632</v>
       </c>
       <c r="B96" s="20" t="s">
         <v>360</v>
@@ -16582,9 +16564,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>638</v>
+        <v>632</v>
       </c>
       <c r="B97" s="20" t="s">
         <v>361</v>
@@ -16729,9 +16711,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>639</v>
+        <v>633</v>
       </c>
       <c r="B98" s="20" t="s">
         <v>362</v>
@@ -16876,9 +16858,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>640</v>
+        <v>634</v>
       </c>
       <c r="B99" s="20" t="s">
         <v>363</v>
@@ -17023,9 +17005,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>642</v>
+        <v>636</v>
       </c>
       <c r="B100" s="20" t="s">
         <v>364</v>
@@ -17170,9 +17152,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>642</v>
+        <v>636</v>
       </c>
       <c r="B101" s="20" t="s">
         <v>365</v>
@@ -17317,9 +17299,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>642</v>
+        <v>636</v>
       </c>
       <c r="B102" s="20" t="s">
         <v>366</v>
@@ -17464,9 +17446,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>641</v>
+        <v>635</v>
       </c>
       <c r="B103" s="20" t="s">
         <v>367</v>
@@ -17611,9 +17593,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>641</v>
+        <v>635</v>
       </c>
       <c r="B104" s="20" t="s">
         <v>368</v>
@@ -17758,9 +17740,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>643</v>
+        <v>637</v>
       </c>
       <c r="B105" s="20" t="s">
         <v>369</v>
@@ -17905,9 +17887,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>643</v>
+        <v>637</v>
       </c>
       <c r="B106" s="20" t="s">
         <v>370</v>
@@ -18052,9 +18034,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>644</v>
+        <v>638</v>
       </c>
       <c r="B107" s="20" t="s">
         <v>371</v>
@@ -18199,9 +18181,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>645</v>
+        <v>639</v>
       </c>
       <c r="B108" s="20" t="s">
         <v>372</v>
@@ -18346,9 +18328,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="B109" s="20" t="s">
         <v>373</v>
@@ -18493,9 +18475,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="B110" s="20" t="s">
         <v>374</v>
@@ -18640,9 +18622,9 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="111" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="B111" s="20" t="s">
         <v>375</v>
@@ -18787,9 +18769,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="B112" s="20" t="s">
         <v>376</v>
@@ -18934,9 +18916,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="B113" s="20" t="s">
         <v>377</v>
@@ -19081,9 +19063,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="B114" s="20" t="s">
         <v>378</v>
@@ -19228,9 +19210,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="B115" s="20" t="s">
         <v>379</v>
@@ -19375,9 +19357,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>647</v>
+        <v>641</v>
       </c>
       <c r="B116" s="20" t="s">
         <v>380</v>
@@ -19522,9 +19504,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="B117" s="4" t="s">
         <v>381</v>
@@ -19669,9 +19651,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="B118" s="4" t="s">
         <v>382</v>
@@ -19816,9 +19798,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="B119" s="4" t="s">
         <v>383</v>
@@ -19963,9 +19945,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="B120" s="4" t="s">
         <v>384</v>
@@ -20110,9 +20092,9 @@
         <v>1032</v>
       </c>
     </row>
-    <row r="121" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="B121" s="4" t="s">
         <v>385</v>
@@ -20257,9 +20239,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>649</v>
+        <v>643</v>
       </c>
       <c r="B122" s="20" t="s">
         <v>386</v>
@@ -20404,9 +20386,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>650</v>
+        <v>644</v>
       </c>
       <c r="B123" s="20" t="s">
         <v>387</v>
@@ -20551,9 +20533,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>651</v>
+        <v>645</v>
       </c>
       <c r="B124" s="20" t="s">
         <v>388</v>
@@ -20698,9 +20680,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>652</v>
+        <v>646</v>
       </c>
       <c r="B125" s="20" t="s">
         <v>389</v>
@@ -20845,9 +20827,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>653</v>
+        <v>647</v>
       </c>
       <c r="B126" s="20" t="s">
         <v>390</v>
@@ -20992,9 +20974,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>653</v>
+        <v>647</v>
       </c>
       <c r="B127" s="20" t="s">
         <v>391</v>
@@ -21139,9 +21121,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>654</v>
+        <v>648</v>
       </c>
       <c r="B128" s="20" t="s">
         <v>392</v>
@@ -21286,9 +21268,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>655</v>
+        <v>649</v>
       </c>
       <c r="B129" s="20" t="s">
         <v>393</v>
@@ -21433,9 +21415,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>655</v>
+        <v>649</v>
       </c>
       <c r="B130" s="20" t="s">
         <v>394</v>
@@ -21580,9 +21562,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>656</v>
+        <v>650</v>
       </c>
       <c r="B131" s="20" t="s">
         <v>395</v>
@@ -21727,9 +21709,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>657</v>
+        <v>651</v>
       </c>
       <c r="B132" s="20" t="s">
         <v>396</v>
@@ -21874,9 +21856,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>657</v>
+        <v>651</v>
       </c>
       <c r="B133" s="20" t="s">
         <v>397</v>
@@ -22021,9 +22003,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>658</v>
+        <v>652</v>
       </c>
       <c r="B134" s="20" t="s">
         <v>398</v>
@@ -22168,9 +22150,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>659</v>
+        <v>653</v>
       </c>
       <c r="B135" s="20" t="s">
         <v>588</v>
@@ -22315,9 +22297,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>660</v>
+        <v>654</v>
       </c>
       <c r="B136" s="20" t="s">
         <v>399</v>
@@ -22462,9 +22444,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>660</v>
+        <v>654</v>
       </c>
       <c r="B137" s="20" t="s">
         <v>399</v>
@@ -22609,9 +22591,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>660</v>
+        <v>654</v>
       </c>
       <c r="B138" s="20" t="s">
         <v>399</v>
@@ -22756,9 +22738,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>661</v>
+        <v>655</v>
       </c>
       <c r="B139" s="20" t="s">
         <v>400</v>
@@ -22903,9 +22885,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>661</v>
+        <v>655</v>
       </c>
       <c r="B140" s="20" t="s">
         <v>401</v>
@@ -23044,9 +23026,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>661</v>
+        <v>655</v>
       </c>
       <c r="B141" s="20" t="s">
         <v>402</v>
@@ -23191,9 +23173,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>661</v>
+        <v>655</v>
       </c>
       <c r="B142" s="20" t="s">
         <v>403</v>
@@ -23332,9 +23314,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>662</v>
+        <v>656</v>
       </c>
       <c r="B143" s="20" t="s">
         <v>404</v>
@@ -23479,9 +23461,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>662</v>
+        <v>656</v>
       </c>
       <c r="B144" s="20" t="s">
         <v>405</v>
@@ -23626,9 +23608,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>662</v>
+        <v>656</v>
       </c>
       <c r="B145" s="20" t="s">
         <v>406</v>
@@ -23773,9 +23755,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>663</v>
+        <v>657</v>
       </c>
       <c r="B146" s="20" t="s">
         <v>407</v>
@@ -23920,9 +23902,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>664</v>
+        <v>658</v>
       </c>
       <c r="B147" s="20" t="s">
         <v>408</v>
@@ -24067,9 +24049,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="B148" s="20" t="s">
         <v>409</v>
@@ -24214,9 +24196,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="B149" s="20" t="s">
         <v>409</v>
@@ -24361,9 +24343,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="B150" s="20" t="s">
         <v>409</v>
@@ -24508,9 +24490,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="B151" s="20" t="s">
         <v>410</v>
@@ -24655,9 +24637,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="B152" s="20" t="s">
         <v>410</v>
@@ -24802,9 +24784,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="B153" s="20" t="s">
         <v>410</v>
@@ -24949,9 +24931,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="B154" s="20" t="s">
         <v>411</v>
@@ -25090,9 +25072,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="B155" s="20" t="s">
         <v>412</v>
@@ -25237,9 +25219,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>665</v>
+        <v>659</v>
       </c>
       <c r="B156" s="20" t="s">
         <v>413</v>
@@ -25384,9 +25366,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>666</v>
+        <v>660</v>
       </c>
       <c r="B157" s="20" t="s">
         <v>414</v>
@@ -25531,9 +25513,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>666</v>
+        <v>660</v>
       </c>
       <c r="B158" s="20" t="s">
         <v>415</v>
@@ -25678,9 +25660,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>666</v>
+        <v>660</v>
       </c>
       <c r="B159" s="20" t="s">
         <v>416</v>
@@ -25825,9 +25807,9 @@
         <v>375</v>
       </c>
     </row>
-    <row r="160" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>667</v>
+        <v>705</v>
       </c>
       <c r="B160" s="20" t="s">
         <v>417</v>
@@ -25972,9 +25954,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>668</v>
+        <v>704</v>
       </c>
       <c r="B161" s="20" t="s">
         <v>417</v>
@@ -26119,9 +26101,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>669</v>
+        <v>661</v>
       </c>
       <c r="B162" s="20" t="s">
         <v>418</v>
@@ -26266,9 +26248,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>670</v>
+        <v>662</v>
       </c>
       <c r="B163" s="20" t="s">
         <v>419</v>
@@ -26413,9 +26395,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>671</v>
+        <v>663</v>
       </c>
       <c r="B164" s="20" t="s">
         <v>420</v>
@@ -26560,9 +26542,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>672</v>
+        <v>664</v>
       </c>
       <c r="B165" s="20" t="s">
         <v>421</v>
@@ -26707,9 +26689,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>673</v>
+        <v>665</v>
       </c>
       <c r="B166" s="20" t="s">
         <v>422</v>
@@ -26854,9 +26836,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>674</v>
+        <v>666</v>
       </c>
       <c r="B167" s="20" t="s">
         <v>423</v>
@@ -27001,9 +26983,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
-        <v>675</v>
+        <v>667</v>
       </c>
       <c r="B168" s="20" t="s">
         <v>424</v>
@@ -27148,9 +27130,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
-        <v>676</v>
+        <v>668</v>
       </c>
       <c r="B169" s="20" t="s">
         <v>425</v>
@@ -27295,9 +27277,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
-        <v>677</v>
+        <v>669</v>
       </c>
       <c r="B170" s="20" t="s">
         <v>426</v>
@@ -27442,9 +27424,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
-        <v>678</v>
+        <v>670</v>
       </c>
       <c r="B171" s="20" t="s">
         <v>427</v>
@@ -27589,9 +27571,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>679</v>
+        <v>671</v>
       </c>
       <c r="B172" s="20" t="s">
         <v>428</v>
@@ -27736,9 +27718,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
-        <v>679</v>
+        <v>671</v>
       </c>
       <c r="B173" s="20" t="s">
         <v>429</v>
@@ -27883,9 +27865,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
-        <v>679</v>
+        <v>671</v>
       </c>
       <c r="B174" s="20" t="s">
         <v>430</v>
@@ -28030,9 +28012,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
-        <v>679</v>
+        <v>671</v>
       </c>
       <c r="B175" s="20" t="s">
         <v>431</v>
@@ -28177,9 +28159,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
-        <v>680</v>
+        <v>672</v>
       </c>
       <c r="B176" s="20" t="s">
         <v>432</v>
@@ -28324,9 +28306,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
-        <v>681</v>
+        <v>673</v>
       </c>
       <c r="B177" s="20" t="s">
         <v>433</v>
@@ -28471,9 +28453,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
-        <v>682</v>
+        <v>674</v>
       </c>
       <c r="B178" s="20" t="s">
         <v>434</v>
@@ -28618,9 +28600,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
-        <v>683</v>
+        <v>675</v>
       </c>
       <c r="B179" s="20" t="s">
         <v>435</v>
@@ -28765,9 +28747,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>684</v>
+        <v>676</v>
       </c>
       <c r="B180" s="20" t="s">
         <v>436</v>
@@ -28912,9 +28894,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
-        <v>685</v>
+        <v>677</v>
       </c>
       <c r="B181" s="20" t="s">
         <v>437</v>
@@ -29059,9 +29041,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
-        <v>685</v>
+        <v>677</v>
       </c>
       <c r="B182" s="20" t="s">
         <v>438</v>
@@ -29206,9 +29188,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
-        <v>686</v>
+        <v>678</v>
       </c>
       <c r="B183" s="20" t="s">
         <v>439</v>
@@ -29353,9 +29335,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
-        <v>687</v>
+        <v>679</v>
       </c>
       <c r="B184" s="20" t="s">
         <v>440</v>
@@ -29500,9 +29482,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
-        <v>687</v>
+        <v>679</v>
       </c>
       <c r="B185" s="20" t="s">
         <v>440</v>
@@ -29647,9 +29629,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
-        <v>687</v>
+        <v>679</v>
       </c>
       <c r="B186" s="20" t="s">
         <v>440</v>
@@ -29794,9 +29776,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
-        <v>688</v>
+        <v>680</v>
       </c>
       <c r="B187" s="20" t="s">
         <v>441</v>
@@ -29941,9 +29923,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
-        <v>689</v>
+        <v>681</v>
       </c>
       <c r="B188" s="20" t="s">
         <v>442</v>
@@ -30088,9 +30070,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
-        <v>690</v>
+        <v>682</v>
       </c>
       <c r="B189" s="20" t="s">
         <v>443</v>
@@ -30235,9 +30217,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
-        <v>691</v>
+        <v>683</v>
       </c>
       <c r="B190" s="20" t="s">
         <v>444</v>
@@ -30382,9 +30364,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
-        <v>692</v>
+        <v>684</v>
       </c>
       <c r="B191" s="20" t="s">
         <v>445</v>
@@ -30529,9 +30511,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
-        <v>692</v>
+        <v>684</v>
       </c>
       <c r="B192" s="20" t="s">
         <v>446</v>
@@ -30676,9 +30658,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
-        <v>693</v>
+        <v>685</v>
       </c>
       <c r="B193" s="20" t="s">
         <v>447</v>
@@ -30823,9 +30805,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
-        <v>693</v>
+        <v>685</v>
       </c>
       <c r="B194" s="20" t="s">
         <v>448</v>
@@ -30970,9 +30952,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="B195" s="20" t="s">
         <v>449</v>
@@ -31117,9 +31099,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="B196" s="20" t="s">
         <v>450</v>
@@ -31264,9 +31246,9 @@
         <v>859</v>
       </c>
     </row>
-    <row r="197" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="B197" s="20" t="s">
         <v>451</v>
@@ -31411,9 +31393,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="B198" s="20" t="s">
         <v>452</v>
@@ -31558,9 +31540,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="B199" s="20" t="s">
         <v>453</v>
@@ -31705,9 +31687,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="B200" s="20" t="s">
         <v>454</v>
@@ -31852,9 +31834,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="B201" s="20" t="s">
         <v>455</v>
@@ -31999,9 +31981,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="B202" s="20" t="s">
         <v>456</v>
@@ -32146,9 +32128,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
-        <v>695</v>
+        <v>687</v>
       </c>
       <c r="B203" s="20" t="s">
         <v>457</v>
@@ -32293,9 +32275,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
-        <v>695</v>
+        <v>687</v>
       </c>
       <c r="B204" s="20" t="s">
         <v>458</v>
@@ -32440,9 +32422,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
-        <v>696</v>
+        <v>688</v>
       </c>
       <c r="B205" s="20" t="s">
         <v>459</v>
@@ -32587,9 +32569,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
-        <v>697</v>
+        <v>689</v>
       </c>
       <c r="B206" s="20" t="s">
         <v>460</v>
@@ -32734,9 +32716,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
-        <v>698</v>
+        <v>690</v>
       </c>
       <c r="B207" s="20" t="s">
         <v>461</v>
@@ -32881,9 +32863,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
-        <v>698</v>
+        <v>690</v>
       </c>
       <c r="B208" s="20" t="s">
         <v>462</v>
@@ -33028,9 +33010,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="B209" s="20" t="s">
         <v>463</v>
@@ -33175,9 +33157,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="B210" s="20" t="s">
         <v>464</v>
@@ -33322,9 +33304,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="B211" s="20" t="s">
         <v>465</v>
@@ -33469,9 +33451,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
-        <v>699</v>
+        <v>691</v>
       </c>
       <c r="B212" s="20" t="s">
         <v>466</v>
@@ -33616,9 +33598,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
-        <v>700</v>
+        <v>692</v>
       </c>
       <c r="B213" s="20" t="s">
         <v>467</v>
@@ -33763,9 +33745,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
-        <v>700</v>
+        <v>692</v>
       </c>
       <c r="B214" s="20" t="s">
         <v>468</v>
@@ -33910,9 +33892,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
-        <v>701</v>
+        <v>693</v>
       </c>
       <c r="B215" s="20" t="s">
         <v>469</v>
@@ -34057,9 +34039,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
-        <v>702</v>
+        <v>694</v>
       </c>
       <c r="B216" s="20" t="s">
         <v>470</v>
@@ -34204,9 +34186,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
-        <v>703</v>
+        <v>695</v>
       </c>
       <c r="B217" s="20" t="s">
         <v>471</v>
@@ -34351,9 +34333,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
-        <v>704</v>
+        <v>696</v>
       </c>
       <c r="B218" s="20" t="s">
         <v>472</v>
@@ -34498,9 +34480,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
-        <v>705</v>
+        <v>697</v>
       </c>
       <c r="B219" s="20" t="s">
         <v>473</v>
@@ -34645,9 +34627,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
-        <v>706</v>
+        <v>698</v>
       </c>
       <c r="B220" s="20" t="s">
         <v>474</v>
@@ -34792,9 +34774,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
-        <v>707</v>
+        <v>699</v>
       </c>
       <c r="B221" s="21" t="s">
         <v>587</v>
@@ -34939,7 +34921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>590</v>
       </c>
@@ -35086,9 +35068,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
-        <v>708</v>
+        <v>700</v>
       </c>
       <c r="B223" s="20" t="s">
         <v>477</v>
@@ -35227,9 +35209,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="B224" s="20" t="s">
         <v>484</v>
@@ -35368,9 +35350,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="B225" s="20" t="s">
         <v>485</v>
@@ -35509,9 +35491,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="B226" s="20" t="s">
         <v>478</v>
@@ -35650,9 +35632,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="B227" s="20" t="s">
         <v>479</v>
@@ -35791,9 +35773,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="B228" s="20" t="s">
         <v>480</v>
@@ -35932,9 +35914,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="B229" s="20" t="s">
         <v>481</v>
@@ -36073,9 +36055,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="B230" s="20" t="s">
         <v>482</v>
@@ -36214,9 +36196,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:49" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:49" ht="18" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="B231" s="20" t="s">
         <v>483</v>

</xml_diff>